<commit_message>
xlstream-eval: fix permut fixture cross-sheet ref and _xlfn. prefix
F2 had cross-sheet PERMUT(Sheet2!A2,Sheet2!B2), replaced with literal.
PERMUTATIONA formulas needed _xlfn. prefix for Excel. Recalculated.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/statistical/permut.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/statistical/permut.xlsx
@@ -1,16 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/statistical/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_BDED0DFC0A0C5F8CA2DF7C7525F1DAD13F69CFAB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -41,8 +60,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,6 +98,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -366,11 +393,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -393,7 +420,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>5</v>
       </c>
@@ -405,7 +432,7 @@
         <v>60</v>
       </c>
       <c r="D2">
-        <f>PERMUTATIONA(5,3)</f>
+        <f>_xlfn.PERMUTATIONA(5,3)</f>
         <v>125</v>
       </c>
       <c r="E2" t="str">
@@ -413,7 +440,7 @@
         <v>many</v>
       </c>
       <c r="F2">
-        <f>PERMUT(Sheet2!A2,Sheet2!B2)</f>
+        <f>PERMUT(8,3)</f>
         <v>336</v>
       </c>
       <c r="G2">
@@ -421,7 +448,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>10</v>
       </c>
@@ -433,7 +460,7 @@
         <v>90</v>
       </c>
       <c r="D3">
-        <f>PERMUTATIONA(3,3)</f>
+        <f>_xlfn.PERMUTATIONA(3,3)</f>
         <v>27</v>
       </c>
       <c r="E3" t="str">
@@ -441,11 +468,11 @@
         <v>invalid</v>
       </c>
       <c r="G3">
-        <f>PERMUTATIONA(2,3)+PERMUT(4,2)</f>
+        <f>_xlfn.PERMUTATIONA(2,3)+PERMUT(4,2)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>0</v>
       </c>
@@ -457,11 +484,11 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <f>PERMUTATIONA(10,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <f>_xlfn.PERMUTATIONA(10,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -473,11 +500,11 @@
         <v>1</v>
       </c>
       <c r="D5">
-        <f>PERMUTATIONA(1,10)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <f>_xlfn.PERMUTATIONA(1,10)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>3</v>
       </c>
@@ -489,11 +516,11 @@
         <v>120</v>
       </c>
       <c r="D6">
-        <f>PERMUTATIONA(0,0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <f>_xlfn.PERMUTATIONA(0,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -505,7 +532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>170</v>
       </c>
@@ -517,7 +544,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C9" t="e">
         <f>PERMUT(3,5)</f>
         <v>#NUM!</v>
@@ -529,11 +556,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -541,7 +568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>8</v>
       </c>

</xml_diff>